<commit_message>
feat : ajout de la planification initiale
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\PlotThoseLines\docs\jdt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F327600-E522-4A5E-BD60-7B12D1FD3FCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D36C95-73D0-420F-9DA6-4E35C05B2945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2790" yWindow="4095" windowWidth="21600" windowHeight="11295" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="37">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -145,10 +145,13 @@
     <t xml:space="preserve">Création des user stories </t>
   </si>
   <si>
-    <t>Création du rapport</t>
+    <t>Amélioration des US</t>
   </si>
   <si>
-    <t>Amélioration des US</t>
+    <t>Création de la planificaiton simple</t>
+  </si>
+  <si>
+    <t>Utiliser un modèle de rapport</t>
   </si>
 </sst>
 </file>
@@ -1156,7 +1159,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>55</c:v>
+                  <c:v>115</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>20</c:v>
@@ -2011,16 +2014,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.6470588235294118</c:v>
+                  <c:v>0.7931034482758621</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.23529411764705882</c:v>
+                  <c:v>0.13793103448275862</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.11764705882352941</c:v>
+                  <c:v>6.8965517241379309E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4255,7 +4258,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>1 heures 25 minutes</v>
+        <v>2 heures 25 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4274,11 +4277,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>85</v>
+        <v>145</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>85</v>
+        <v>145</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4377,7 +4380,7 @@
         <v>17</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G9" s="40"/>
       <c r="M9" t="s">
@@ -4406,7 +4409,7 @@
         <v>14</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G10" s="39"/>
       <c r="M10" t="s">
@@ -4420,15 +4423,23 @@
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="63" t="str">
+      <c r="A11" s="63">
         <f>IF(ISBLANK(B11),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B11))</f>
-        <v/>
-      </c>
-      <c r="B11" s="34"/>
+        <v>36</v>
+      </c>
+      <c r="B11" s="34">
+        <v>46265</v>
+      </c>
       <c r="C11" s="35"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="37"/>
-      <c r="F11" s="23"/>
+      <c r="D11" s="36">
+        <v>20</v>
+      </c>
+      <c r="E11" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>35</v>
+      </c>
       <c r="G11" s="40"/>
       <c r="M11" t="s">
         <v>17</v>
@@ -4441,15 +4452,23 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="62" t="str">
+      <c r="A12" s="62">
         <f>IF(ISBLANK(B12),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B12))</f>
-        <v/>
-      </c>
-      <c r="B12" s="30"/>
+        <v>36</v>
+      </c>
+      <c r="B12" s="30">
+        <v>46265</v>
+      </c>
       <c r="C12" s="31"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="23"/>
+      <c r="D12" s="32">
+        <v>40</v>
+      </c>
+      <c r="E12" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>34</v>
+      </c>
       <c r="G12" s="39"/>
       <c r="M12" t="s">
         <v>18</v>
@@ -10869,11 +10888,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>55</v>
+        <v>115</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>55</v>
+        <v>115</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10881,11 +10900,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>0 h 55 min</v>
+        <v>1 h 55 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.6470588235294118</v>
+        <v>0.7931034482758621</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10922,7 +10941,7 @@
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.23529411764705882</v>
+        <v>0.13793103448275862</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10996,7 +11015,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.11764705882352941</v>
+        <v>6.8965517241379309E-2</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11052,22 +11071,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>85</v>
+        <v>145</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>85</v>
+        <v>145</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>1 h 25 min</v>
+        <v>2 h 25 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>1.5740740740740739E-2</v>
+        <v>2.6851851851851852E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11106,6 +11125,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="62349bcdb43c26c508700efba1cb50b1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e5d6db3f342a25e0e30f4a2965162e1" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11294,41 +11333,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11351,9 +11359,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat : màj jdt + ajout d'analyse fonctionnelle
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\PlotThoseLines\docs\jdt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D36C95-73D0-420F-9DA6-4E35C05B2945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA64B518-5CEB-458F-9A9E-8B7A027EF8EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2790" yWindow="4095" windowWidth="21600" windowHeight="11295" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="39">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -152,6 +152,12 @@
   </si>
   <si>
     <t>Utiliser un modèle de rapport</t>
+  </si>
+  <si>
+    <t>Création de la maquette</t>
+  </si>
+  <si>
+    <t>Ajout de tests d'acceptence à chaque fois, image de la maquette, US atomiques</t>
   </si>
 </sst>
 </file>
@@ -1159,7 +1165,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>115</c:v>
+                  <c:v>145</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>20</c:v>
@@ -2014,16 +2020,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.7931034482758621</c:v>
+                  <c:v>0.82857142857142863</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.13793103448275862</c:v>
+                  <c:v>0.11428571428571428</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>6.8965517241379309E-2</c:v>
+                  <c:v>5.7142857142857141E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4258,7 +4264,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>2 heures 25 minutes</v>
+        <v>2 heures 55 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4277,11 +4283,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>145</v>
+        <v>175</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>145</v>
+        <v>175</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4461,13 +4467,13 @@
       </c>
       <c r="C12" s="31"/>
       <c r="D12" s="32">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E12" s="33" t="s">
         <v>14</v>
       </c>
       <c r="F12" s="23" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="G12" s="39"/>
       <c r="M12" t="s">
@@ -4481,16 +4487,26 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="63" t="str">
+      <c r="A13" s="63">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
-        <v/>
-      </c>
-      <c r="B13" s="34"/>
+        <v>36</v>
+      </c>
+      <c r="B13" s="34">
+        <v>46265</v>
+      </c>
       <c r="C13" s="35"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="40"/>
+      <c r="D13" s="36">
+        <v>40</v>
+      </c>
+      <c r="E13" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="G13" s="40" t="s">
+        <v>38</v>
+      </c>
       <c r="N13">
         <v>6</v>
       </c>
@@ -10888,11 +10904,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>115</v>
+        <v>145</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>115</v>
+        <v>145</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10900,11 +10916,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>1 h 55 min</v>
+        <v>2 h 25 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.7931034482758621</v>
+        <v>0.82857142857142863</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10941,7 +10957,7 @@
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.13793103448275862</v>
+        <v>0.11428571428571428</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11015,7 +11031,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>6.8965517241379309E-2</v>
+        <v>5.7142857142857141E-2</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11071,22 +11087,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>145</v>
+        <v>175</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>145</v>
+        <v>175</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>2 h 25 min</v>
+        <v>2 h 55 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>2.6851851851851852E-2</v>
+        <v>3.2407407407407406E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
feat : ajout des classes DataPoint et DataSerie
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\PlotThoseLines\docs\jdt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{578EC55F-2D92-4FD8-9DB8-DBFA6C3F81A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF524128-86C3-4E1F-AA1D-9BE32814B409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2790" yWindow="4095" windowWidth="21600" windowHeight="11295" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -1180,7 +1180,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>40</c:v>
+                  <c:v>55</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2026,16 +2026,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.70731707317073167</c:v>
+                  <c:v>0.65909090909090906</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>9.7560975609756101E-2</c:v>
+                  <c:v>9.0909090909090912E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.1951219512195122</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4270,7 +4270,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>3 heures 25 minutes</v>
+        <v>3 heures 40 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4289,11 +4289,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4530,7 +4530,7 @@
       </c>
       <c r="C14" s="31"/>
       <c r="D14" s="32">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="E14" s="33" t="s">
         <v>17</v>
@@ -10831,7 +10831,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="52" orientation="landscape" r:id="rId1"/>
   <tableParts count="1">
     <tablePart r:id="rId2"/>
   </tableParts>
@@ -10936,7 +10936,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.70731707317073167</v>
+        <v>0.65909090909090906</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10973,7 +10973,7 @@
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>9.7560975609756101E-2</v>
+        <v>9.0909090909090912E-2</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11031,11 +11031,11 @@
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11043,11 +11043,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>0 h 40 min</v>
+        <v>0 h 55 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.1951219512195122</v>
+        <v>0.25</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11103,22 +11103,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>3 h 25 min</v>
+        <v>3 h 40 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>3.7962962962962962E-2</v>
+        <v>4.0740740740740744E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11141,7 +11141,8 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="u6Q3+o7a9rb9ajPGMQFXFJBxNR95C93y6qzzKCld0gZtCTYGL+7OMe+WbK2ki7xwzk+WSRqA9/xPSrIc7CBoPg==" saltValue="e1RdssACZUGVypOFgaRLDA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -11152,7 +11153,8 @@
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="hkKOZ8xr/Okjo/AJlNTtoGYYhES8sIn2fOpGKGGyPJqhNRzaMuj9V6Pke+VqLSypQTwaNPCt0dhRPEVp9CfBFA==" saltValue="lF/ApQWS3LBdJp0wgcNUcQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -11376,16 +11378,16 @@
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
docs : màj jdt et rapport
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\PlotThoseLines\docs\jdt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF524128-86C3-4E1F-AA1D-9BE32814B409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8361483A-B181-498B-8A97-74560A03622D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2790" yWindow="4095" windowWidth="21600" windowHeight="11295" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="34395" yWindow="840" windowWidth="21600" windowHeight="13305" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="53">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -164,6 +164,42 @@
   </si>
   <si>
     <t>J'ai ajouté les sections description, objectifs, analyse fonctionnelle et planificaiton simple</t>
+  </si>
+  <si>
+    <t>Daily Scrum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyse de travail fait la dernière fois, j'ai fini avec les US, l'into du rapport et la planification, aujourd'hui je m'attaque au code </t>
+  </si>
+  <si>
+    <t>Ajout du composant ScottPlot dans le projet</t>
+  </si>
+  <si>
+    <t>Écriture du fichier DataPoint</t>
+  </si>
+  <si>
+    <t>Création du fichier DataSerie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai dû passer beaucoup de temps sur la création de ce composant, en décorticant chaque ligne, parce que initialement j'ai pas très bien compris le concept </t>
+  </si>
+  <si>
+    <t>Introduction dans la journée par le chef du projet</t>
+  </si>
+  <si>
+    <t>Introduction au projet par le chef du projet</t>
+  </si>
+  <si>
+    <t>Le Chef du projet a expliqué les buts du projet et le déroulement</t>
+  </si>
+  <si>
+    <t>Informations supplémentaires par le chef de projet</t>
+  </si>
+  <si>
+    <t>Test de ScottPlot avec des données fausses</t>
+  </si>
+  <si>
+    <t>Feedback de chef de projet par rapport au US, rapport et jdt</t>
   </si>
 </sst>
 </file>
@@ -1171,10 +1207,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>145</c:v>
+                  <c:v>310</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>20</c:v>
+                  <c:v>140</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2026,16 +2062,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.65909090909090906</c:v>
+                  <c:v>0.61386138613861385</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>9.0909090909090912E-2</c:v>
+                  <c:v>0.27722772277227725</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.25</c:v>
+                  <c:v>0.10891089108910891</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4270,7 +4306,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>3 heures 40 minutes</v>
+        <v>8 heures 25 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4285,15 +4321,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>220</v>
+        <v>385</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>220</v>
+        <v>505</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4335,17 +4371,21 @@
       <c r="B7" s="26">
         <v>46258</v>
       </c>
-      <c r="C7" s="27"/>
+      <c r="C7" s="27">
+        <v>1</v>
+      </c>
       <c r="D7" s="28">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="G7" s="38"/>
+        <v>48</v>
+      </c>
+      <c r="G7" s="38" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="62">
@@ -4357,13 +4397,13 @@
       </c>
       <c r="C8" s="31"/>
       <c r="D8" s="32">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F8" s="23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G8" s="39"/>
       <c r="M8" t="s">
@@ -4386,13 +4426,13 @@
       </c>
       <c r="C9" s="35"/>
       <c r="D9" s="36">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G9" s="40"/>
       <c r="M9" t="s">
@@ -4415,13 +4455,13 @@
       </c>
       <c r="C10" s="31"/>
       <c r="D10" s="32">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G10" s="39"/>
       <c r="M10" t="s">
@@ -4437,20 +4477,20 @@
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="63">
         <f>IF(ISBLANK(B11),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B11))</f>
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B11" s="34">
-        <v>46265</v>
+        <v>46258</v>
       </c>
       <c r="C11" s="35"/>
       <c r="D11" s="36">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E11" s="37" t="s">
         <v>14</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G11" s="40"/>
       <c r="M11" t="s">
@@ -4473,13 +4513,13 @@
       </c>
       <c r="C12" s="31"/>
       <c r="D12" s="32">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E12" s="33" t="s">
         <v>14</v>
       </c>
       <c r="F12" s="23" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="G12" s="39"/>
       <c r="M12" t="s">
@@ -4502,17 +4542,15 @@
       </c>
       <c r="C13" s="35"/>
       <c r="D13" s="36">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="E13" s="37" t="s">
         <v>14</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="G13" s="40" t="s">
-        <v>38</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="G13" s="40"/>
       <c r="N13">
         <v>6</v>
       </c>
@@ -4530,17 +4568,15 @@
       </c>
       <c r="C14" s="31"/>
       <c r="D14" s="32">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="G14" s="39" t="s">
-        <v>40</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="G14" s="39"/>
       <c r="N14">
         <v>7</v>
       </c>
@@ -4549,15 +4585,23 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="63" t="str">
+      <c r="A15" s="63">
         <f>IF(ISBLANK(B15),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B15))</f>
-        <v/>
-      </c>
-      <c r="B15" s="34"/>
+        <v>36</v>
+      </c>
+      <c r="B15" s="34">
+        <v>46265</v>
+      </c>
       <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="23"/>
+      <c r="D15" s="36">
+        <v>40</v>
+      </c>
+      <c r="E15" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>37</v>
+      </c>
       <c r="G15" s="40"/>
       <c r="N15">
         <v>8</v>
@@ -4567,123 +4611,203 @@
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="62" t="str">
+      <c r="A16" s="62">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
-        <v/>
-      </c>
-      <c r="B16" s="30"/>
+        <v>36</v>
+      </c>
+      <c r="B16" s="30">
+        <v>46265</v>
+      </c>
       <c r="C16" s="31"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="39"/>
+      <c r="D16" s="32">
+        <v>40</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="G16" s="39" t="s">
+        <v>38</v>
+      </c>
       <c r="O16">
         <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="63" t="str">
+      <c r="A17" s="63">
         <f>IF(ISBLANK(B17),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B17))</f>
-        <v/>
-      </c>
-      <c r="B17" s="34"/>
+        <v>36</v>
+      </c>
+      <c r="B17" s="34">
+        <v>46265</v>
+      </c>
       <c r="C17" s="35"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="40"/>
+      <c r="D17" s="36">
+        <v>45</v>
+      </c>
+      <c r="E17" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="G17" s="40" t="s">
+        <v>40</v>
+      </c>
       <c r="O17">
         <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="62" t="str">
+      <c r="A18" s="62">
         <f>IF(ISBLANK(B18),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B18))</f>
-        <v/>
-      </c>
-      <c r="B18" s="30"/>
+        <v>37</v>
+      </c>
+      <c r="B18" s="30">
+        <v>46272</v>
+      </c>
       <c r="C18" s="31"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="23"/>
+      <c r="D18" s="32">
+        <v>10</v>
+      </c>
+      <c r="E18" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>47</v>
+      </c>
       <c r="G18" s="39"/>
       <c r="O18">
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="63" t="str">
+    <row r="19" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A19" s="63">
         <f>IF(ISBLANK(B19),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B19))</f>
-        <v/>
-      </c>
-      <c r="B19" s="34"/>
+        <v>37</v>
+      </c>
+      <c r="B19" s="34">
+        <v>46272</v>
+      </c>
       <c r="C19" s="35"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="40"/>
+      <c r="D19" s="36">
+        <v>10</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="G19" s="40" t="s">
+        <v>42</v>
+      </c>
       <c r="O19">
         <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="62" t="str">
+      <c r="A20" s="62">
         <f>IF(ISBLANK(B20),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B20))</f>
-        <v/>
-      </c>
-      <c r="B20" s="30"/>
+        <v>37</v>
+      </c>
+      <c r="B20" s="30">
+        <v>46272</v>
+      </c>
       <c r="C20" s="31"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="23"/>
+      <c r="D20" s="32">
+        <v>10</v>
+      </c>
+      <c r="E20" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>43</v>
+      </c>
       <c r="G20" s="39"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="63" t="str">
+      <c r="A21" s="63">
         <f>IF(ISBLANK(B21),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B21))</f>
-        <v/>
-      </c>
-      <c r="B21" s="34"/>
+        <v>37</v>
+      </c>
+      <c r="B21" s="34">
+        <v>46272</v>
+      </c>
       <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="23"/>
+      <c r="D21" s="36">
+        <v>20</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>44</v>
+      </c>
       <c r="G21" s="40"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="62" t="str">
+      <c r="A22" s="62">
         <f>IF(ISBLANK(B22),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B22))</f>
-        <v/>
-      </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="31"/>
+        <v>37</v>
+      </c>
+      <c r="B22" s="30">
+        <v>46272</v>
+      </c>
+      <c r="C22" s="31">
+        <v>1</v>
+      </c>
       <c r="D22" s="32"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="23"/>
-      <c r="G22" s="39"/>
+      <c r="E22" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="G22" s="39" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="63" t="str">
+      <c r="A23" s="63">
         <f>IF(ISBLANK(B23),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B23))</f>
-        <v/>
-      </c>
-      <c r="B23" s="34"/>
+        <v>37</v>
+      </c>
+      <c r="B23" s="34">
+        <v>46272</v>
+      </c>
       <c r="C23" s="35"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="23"/>
+      <c r="D23" s="36">
+        <v>30</v>
+      </c>
+      <c r="E23" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="23" t="s">
+        <v>51</v>
+      </c>
       <c r="G23" s="40"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="62" t="str">
+      <c r="A24" s="62">
         <f>IF(ISBLANK(B24),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B24))</f>
-        <v/>
-      </c>
-      <c r="B24" s="30"/>
+        <v>37</v>
+      </c>
+      <c r="B24" s="30">
+        <v>46272</v>
+      </c>
       <c r="C24" s="31"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="23"/>
+      <c r="D24" s="32">
+        <v>10</v>
+      </c>
+      <c r="E24" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" s="23" t="s">
+        <v>52</v>
+      </c>
       <c r="G24" s="39"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -10916,15 +11040,15 @@
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>145</v>
+        <v>250</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>145</v>
+        <v>310</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10932,11 +11056,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>2 h 25 min</v>
+        <v>5 h 10 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.65909090909090906</v>
+        <v>0.61386138613861385</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10953,15 +11077,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>140</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10969,11 +11093,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>0 h 20 min</v>
+        <v>2 h 20 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>9.0909090909090912E-2</v>
+        <v>0.27722772277227725</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11047,7 +11171,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.25</v>
+        <v>0.10891089108910891</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11099,26 +11223,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>220</v>
+        <v>385</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>220</v>
+        <v>505</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>3 h 40 min</v>
+        <v>8 h 25 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>4.0740740740740744E-2</v>
+        <v>9.3518518518518515E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11159,26 +11283,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="62349bcdb43c26c508700efba1cb50b1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e5d6db3f342a25e0e30f4a2965162e1" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11367,10 +11471,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11393,20 +11528,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat : ajout de composant pour import des data [WIP]
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\PlotThoseLines\docs\jdt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8361483A-B181-498B-8A97-74560A03622D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4867856C-56A7-4626-95B6-414629032E98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34395" yWindow="840" windowWidth="21600" windowHeight="13305" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="3885" yWindow="1830" windowWidth="21600" windowHeight="13305" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="56">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -200,6 +200,15 @@
   </si>
   <si>
     <t>Feedback de chef de projet par rapport au US, rapport et jdt</t>
+  </si>
+  <si>
+    <t>Remplissage du jdt</t>
+  </si>
+  <si>
+    <t>Correction du rapport + ajout d'infos dans la section bilan de planification</t>
+  </si>
+  <si>
+    <t>Recherche de fichiers avec les données</t>
   </si>
 </sst>
 </file>
@@ -1207,16 +1216,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>310</c:v>
+                  <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>140</c:v>
+                  <c:v>310</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>55</c:v>
+                  <c:v>70</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2062,16 +2071,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.61386138613861385</c:v>
+                  <c:v>0.28301886792452829</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.27722772277227725</c:v>
+                  <c:v>0.58490566037735847</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.10891089108910891</c:v>
+                  <c:v>0.13207547169811321</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4306,7 +4315,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>8 heures 25 minutes</v>
+        <v>8 heures 50 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4325,11 +4334,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>385</v>
+        <v>410</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>505</v>
+        <v>530</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4429,7 +4438,7 @@
         <v>40</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F9" s="23" t="s">
         <v>33</v>
@@ -4487,7 +4496,7 @@
         <v>15</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F11" s="23" t="s">
         <v>34</v>
@@ -4571,7 +4580,7 @@
         <v>25</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F14" s="23" t="s">
         <v>35</v>
@@ -4597,7 +4606,7 @@
         <v>40</v>
       </c>
       <c r="E15" s="37" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F15" s="23" t="s">
         <v>37</v>
@@ -4623,7 +4632,7 @@
         <v>40</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F16" s="23" t="s">
         <v>34</v>
@@ -4811,39 +4820,63 @@
       <c r="G24" s="39"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="63" t="str">
+      <c r="A25" s="63">
         <f>IF(ISBLANK(B25),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B25))</f>
-        <v/>
-      </c>
-      <c r="B25" s="34"/>
+        <v>37</v>
+      </c>
+      <c r="B25" s="34">
+        <v>46272</v>
+      </c>
       <c r="C25" s="35"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="23"/>
+      <c r="D25" s="36">
+        <v>5</v>
+      </c>
+      <c r="E25" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>53</v>
+      </c>
       <c r="G25" s="40"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="62" t="str">
+      <c r="A26" s="62">
         <f>IF(ISBLANK(B26),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B26))</f>
-        <v/>
-      </c>
-      <c r="B26" s="30"/>
+        <v>37</v>
+      </c>
+      <c r="B26" s="30">
+        <v>46272</v>
+      </c>
       <c r="C26" s="31"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="23"/>
+      <c r="D26" s="32">
+        <v>10</v>
+      </c>
+      <c r="E26" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F26" s="23" t="s">
+        <v>54</v>
+      </c>
       <c r="G26" s="39"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="63" t="str">
+      <c r="A27" s="63">
         <f>IF(ISBLANK(B27),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B27))</f>
-        <v/>
-      </c>
-      <c r="B27" s="34"/>
+        <v>37</v>
+      </c>
+      <c r="B27" s="34">
+        <v>46272</v>
+      </c>
       <c r="C27" s="35"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="37"/>
-      <c r="F27" s="23"/>
+      <c r="D27" s="36">
+        <v>10</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F27" s="23" t="s">
+        <v>55</v>
+      </c>
       <c r="G27" s="40"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
@@ -11044,11 +11077,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>250</v>
+        <v>90</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>310</v>
+        <v>150</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11056,11 +11089,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>5 h 10 min</v>
+        <v>2 h 30 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.61386138613861385</v>
+        <v>0.28301886792452829</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11081,11 +11114,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>80</v>
+        <v>250</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>140</v>
+        <v>310</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11093,11 +11126,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>2 h 20 min</v>
+        <v>5 h 10 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.27722772277227725</v>
+        <v>0.58490566037735847</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11155,11 +11188,11 @@
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11167,11 +11200,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>0 h 55 min</v>
+        <v>1 h 10 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.10891089108910891</v>
+        <v>0.13207547169811321</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11227,22 +11260,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>385</v>
+        <v>410</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>505</v>
+        <v>530</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>8 h 25 min</v>
+        <v>8 h 50 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>9.3518518518518515E-2</v>
+        <v>9.8148148148148151E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>

</xml_diff>